<commit_message>
Update applicant import template fields
</commit_message>
<xml_diff>
--- a/求职者信息快速录入模板.xlsx
+++ b/求职者信息快速录入模板.xlsx
@@ -43,7 +43,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q100"/>
+  <dimension ref="A1:S100"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -51,7 +51,7 @@
     <col min="3" max="4" width="10" customWidth="1"/>
     <col min="5" max="9" width="16" customWidth="1"/>
     <col min="10" max="11" width="28" customWidth="1"/>
-    <col min="12" max="17" width="16" customWidth="1"/>
+    <col min="12" max="19" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -140,8 +140,18 @@
           <t>健康/体检情况</t>
         </is>
       </c>
+      <c r="R" t="inlineStr">
+        <is>
+          <t>服务状态</t>
+        </is>
+      </c>
+      <c r="S" t="inlineStr">
+        <is>
+          <t>下次跟进日期</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q100"/>
+  <autoFilter ref="A1:S100"/>
 </worksheet>
 </file>
</xml_diff>